<commit_message>
Add proper thick borders and real reference fields to all templates
Reviewed the actual Word/Excel reference templates (not just the PDFs
checked earlier) and found two real gaps: our borders were too thin/
subtle compared to the fill-in-form convention real quotation templates
use, and we were missing fields present in every reference sample
(Description of Work section, SGST/CGST split instead of flat GST,
Amount in Words, a Discount line).

- PDF: Bold/Formal/Compact themes now use a visible GRID border around
  every cell (Minimal intentionally keeps its thin-rule look, as the
  one deliberately understated option among four).
- Word/Excel: full thick-bordered boxes throughout, Description of Work
  field added, GST split into SGST+CGST (matches real Indian
  convention), Discount line and Amount in Words field added.
- Regenerated all 6 gallery thumbnails from the updated files.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/templates/billbolo-quotation-format.xlsx
+++ b/assets/templates/billbolo-quotation-format.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -41,7 +41,7 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="0094A3B8"/>
+      <color rgb="00FFFFFF"/>
       <sz val="9"/>
     </font>
     <font>
@@ -60,6 +60,10 @@
       <b val="1"/>
       <color rgb="000284C7"/>
       <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="9"/>
     </font>
     <font>
       <b val="1"/>
@@ -83,7 +87,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -92,15 +96,136 @@
       <diagonal/>
     </border>
     <border>
+      <left style="medium">
+        <color rgb="000F172A"/>
+      </left>
+      <right style="thin">
+        <color rgb="0094A3B8"/>
+      </right>
+      <top style="medium">
+        <color rgb="000F172A"/>
+      </top>
       <bottom style="thin">
-        <color rgb="00E2E8F0"/>
+        <color rgb="0094A3B8"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="0094A3B8"/>
+      </left>
+      <right style="thin">
+        <color rgb="0094A3B8"/>
+      </right>
+      <top style="medium">
+        <color rgb="000F172A"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="0094A3B8"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="0094A3B8"/>
+      </left>
+      <right style="medium">
+        <color rgb="000F172A"/>
+      </right>
+      <top style="medium">
+        <color rgb="000F172A"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="0094A3B8"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="000F172A"/>
+      </left>
+      <right style="thin">
+        <color rgb="0094A3B8"/>
+      </right>
+      <top style="thin">
+        <color rgb="0094A3B8"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="0094A3B8"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="0094A3B8"/>
+      </left>
+      <right style="thin">
+        <color rgb="0094A3B8"/>
+      </right>
+      <top style="thin">
+        <color rgb="0094A3B8"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="0094A3B8"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="0094A3B8"/>
+      </left>
+      <right style="medium">
+        <color rgb="000F172A"/>
+      </right>
+      <top style="thin">
+        <color rgb="0094A3B8"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="0094A3B8"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="000F172A"/>
+      </left>
+      <right style="thin">
+        <color rgb="0094A3B8"/>
+      </right>
+      <top style="thin">
+        <color rgb="0094A3B8"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="000F172A"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="0094A3B8"/>
+      </left>
+      <right style="thin">
+        <color rgb="0094A3B8"/>
+      </right>
+      <top style="thin">
+        <color rgb="0094A3B8"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="000F172A"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="0094A3B8"/>
+      </left>
+      <right style="medium">
+        <color rgb="000F172A"/>
+      </right>
+      <top style="thin">
+        <color rgb="0094A3B8"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="000F172A"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -112,24 +237,42 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -495,14 +638,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -521,7 +664,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>[Your Phone Number]</t>
+          <t>[Address]</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
@@ -536,6 +679,11 @@
       </c>
     </row>
     <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>[Your Phone Number]   GSTIN: [Your GSTIN]</t>
+        </is>
+      </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Date:</t>
@@ -553,176 +701,259 @@
           <t>BILL TO</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="B6" s="6" t="n"/>
+      <c r="C6" s="7" t="n"/>
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>VALID UNTIL</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="E6" s="7" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>[Client Name]</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="n"/>
+      <c r="C7" s="10" t="n"/>
+      <c r="D7" s="11" t="inlineStr">
         <is>
           <t>[DD/MM/YYYY]</t>
         </is>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>[Client Name]</t>
-        </is>
-      </c>
+      <c r="E7" s="10" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>[Client Address]</t>
         </is>
       </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="8" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B10" s="8" t="inlineStr">
-        <is>
-          <t>Qty</t>
-        </is>
-      </c>
-      <c r="C10" s="8" t="inlineStr">
-        <is>
-          <t>Rate (Rs.)</t>
-        </is>
-      </c>
-      <c r="D10" s="8" t="inlineStr">
-        <is>
-          <t>Unit</t>
-        </is>
-      </c>
-      <c r="E10" s="8" t="inlineStr">
-        <is>
-          <t>Amount (Rs.)</t>
-        </is>
-      </c>
+      <c r="B8" s="9" t="n"/>
+      <c r="C8" s="10" t="n"/>
+      <c r="D8" s="12" t="n"/>
+      <c r="E8" s="10" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>GSTIN: [Client GSTIN, if applicable]</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="n"/>
+      <c r="C9" s="15" t="n"/>
+      <c r="D9" s="13" t="n"/>
+      <c r="E9" s="15" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="n"/>
-      <c r="B11" s="9" t="n"/>
-      <c r="C11" s="9" t="n"/>
-      <c r="D11" s="9" t="n"/>
-      <c r="E11" s="9">
-        <f>IF(AND(ISNUMBER(B11),ISNUMBER(C11)),B11*C11,"")</f>
-        <v/>
-      </c>
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>DESCRIPTION OF WORK</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="n"/>
+      <c r="C11" s="6" t="n"/>
+      <c r="D11" s="6" t="n"/>
+      <c r="E11" s="7" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="9" t="n"/>
+      <c r="A12" s="12" t="n"/>
       <c r="B12" s="9" t="n"/>
       <c r="C12" s="9" t="n"/>
       <c r="D12" s="9" t="n"/>
-      <c r="E12" s="9">
-        <f>IF(AND(ISNUMBER(B12),ISNUMBER(C12)),B12*C12,"")</f>
-        <v/>
-      </c>
+      <c r="E12" s="10" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="9" t="n"/>
-      <c r="B13" s="9" t="n"/>
-      <c r="C13" s="9" t="n"/>
-      <c r="D13" s="9" t="n"/>
-      <c r="E13" s="9">
-        <f>IF(AND(ISNUMBER(B13),ISNUMBER(C13)),B13*C13,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="9" t="n"/>
-      <c r="B14" s="9" t="n"/>
-      <c r="C14" s="9" t="n"/>
-      <c r="D14" s="9" t="n"/>
-      <c r="E14" s="9">
-        <f>IF(AND(ISNUMBER(B14),ISNUMBER(C14)),B14*C14,"")</f>
-        <v/>
-      </c>
+      <c r="A13" s="13" t="n"/>
+      <c r="B13" s="14" t="n"/>
+      <c r="C13" s="14" t="n"/>
+      <c r="D13" s="14" t="n"/>
+      <c r="E13" s="15" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="9" t="n"/>
-      <c r="B15" s="9" t="n"/>
-      <c r="C15" s="9" t="n"/>
-      <c r="D15" s="9" t="n"/>
-      <c r="E15" s="9">
-        <f>IF(AND(ISNUMBER(B15),ISNUMBER(C15)),B15*C15,"")</f>
-        <v/>
+      <c r="A15" s="16" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B15" s="17" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="C15" s="17" t="inlineStr">
+        <is>
+          <t>Rate (Rs.)</t>
+        </is>
+      </c>
+      <c r="D15" s="17" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="E15" s="18" t="inlineStr">
+        <is>
+          <t>Amount (Rs.)</t>
+        </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="9" t="n"/>
+      <c r="A16" s="12" t="n"/>
       <c r="B16" s="9" t="n"/>
       <c r="C16" s="9" t="n"/>
       <c r="D16" s="9" t="n"/>
-      <c r="E16" s="9">
+      <c r="E16" s="10">
         <f>IF(AND(ISNUMBER(B16),ISNUMBER(C16)),B16*C16,"")</f>
         <v/>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="12" t="n"/>
+      <c r="B17" s="9" t="n"/>
+      <c r="C17" s="9" t="n"/>
+      <c r="D17" s="9" t="n"/>
+      <c r="E17" s="10">
+        <f>IF(AND(ISNUMBER(B17),ISNUMBER(C17)),B17*C17,"")</f>
+        <v/>
+      </c>
+    </row>
     <row r="18">
-      <c r="D18" s="10" t="inlineStr">
+      <c r="A18" s="12" t="n"/>
+      <c r="B18" s="9" t="n"/>
+      <c r="C18" s="9" t="n"/>
+      <c r="D18" s="9" t="n"/>
+      <c r="E18" s="10">
+        <f>IF(AND(ISNUMBER(B18),ISNUMBER(C18)),B18*C18,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="n"/>
+      <c r="B19" s="9" t="n"/>
+      <c r="C19" s="9" t="n"/>
+      <c r="D19" s="9" t="n"/>
+      <c r="E19" s="10">
+        <f>IF(AND(ISNUMBER(B19),ISNUMBER(C19)),B19*C19,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="12" t="n"/>
+      <c r="B20" s="9" t="n"/>
+      <c r="C20" s="9" t="n"/>
+      <c r="D20" s="9" t="n"/>
+      <c r="E20" s="10">
+        <f>IF(AND(ISNUMBER(B20),ISNUMBER(C20)),B20*C20,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="13" t="n"/>
+      <c r="B21" s="14" t="n"/>
+      <c r="C21" s="14" t="n"/>
+      <c r="D21" s="14" t="n"/>
+      <c r="E21" s="15">
+        <f>IF(AND(ISNUMBER(B21),ISNUMBER(C21)),B21*C21,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="D23" s="19" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="E18">
-        <f>SUM(E11:E16)</f>
+      <c r="E23" s="20">
+        <f>SUM(E16:E21)</f>
         <v/>
       </c>
     </row>
-    <row r="19">
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>GST @ 18%</t>
-        </is>
-      </c>
-      <c r="E19">
-        <f>E18*0.18</f>
+    <row r="24">
+      <c r="D24" s="21" t="inlineStr">
+        <is>
+          <t>SGST @ 9%</t>
+        </is>
+      </c>
+      <c r="E24" s="10">
+        <f>E23*0.09</f>
         <v/>
       </c>
     </row>
-    <row r="20">
-      <c r="D20" s="11" t="inlineStr">
+    <row r="25">
+      <c r="D25" s="21" t="inlineStr">
+        <is>
+          <t>CGST @ 9%</t>
+        </is>
+      </c>
+      <c r="E25" s="10">
+        <f>E23*0.09</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="D26" s="21" t="inlineStr">
+        <is>
+          <t>Discount</t>
+        </is>
+      </c>
+      <c r="E26" s="10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="D27" s="22" t="inlineStr">
         <is>
           <t>Grand Total</t>
         </is>
       </c>
-      <c r="E20" s="12">
-        <f>E18+E19</f>
+      <c r="E27" s="23">
+        <f>E23+E24+E25-E26</f>
         <v/>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="13" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="24" t="inlineStr">
+        <is>
+          <t>Amount in Words:</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>[Rupees ... Only]</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="25" t="inlineStr">
         <is>
           <t>Terms &amp; Conditions</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
         <is>
           <t>Valid for 15 days from date of issue. Payment terms to be confirmed before work begins.</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="14" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="26" t="inlineStr">
         <is>
           <t>Free quotation format by BillBolo — billbolo.in</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="6">
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="A12:E13"/>
     <mergeCell ref="A1:C2"/>
     <mergeCell ref="D1:E2"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="A11:E11"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>